<commit_message>
[OOO][DATA] D01-F0-W6 sub-model a formal-385 backfilled
formal_D01-F0-W6-a (opcode_bitflip/transient_bit_flip@coremark) 完成:
385/385 valid(r0000-r0384 完整,385×f=1),Masked 243/Crash 142/SDC 0,
P_DUE 36.9%[32.2,41.8](pilot 30% 一致)。行=预登记重点,现记 385 层,
2401 扩样待 b/c/d 齐后规划;Z=部分证据(W6 仅 CoreMark+b/c/d 未跑)。
16 单元格变更,六步协议核验 ALL PASS(sheets/310 RunID/公式/AM 守恒)。
16 单元格变更对应 row3,备份 bak-20261012-133146。
</commit_message>
<xml_diff>
--- a/docs/gem5-fi/ooo/gem5-fi-OOO单元故障注入方案.xlsx
+++ b/docs/gem5-fi/ooo/gem5-fi-OOO单元故障注入方案.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="12">
     <font>
       <name val="Carlito"/>
@@ -201,7 +203,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
@@ -315,6 +317,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -771,7 +779,7 @@
     <row r="24" ht="72" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>6) 最终结局分为 Masked、Detected-contained、Data Corruption、Crash、Timeout；SDC = 运行时三层均未检测且正常完成，但离线 oracle 发现 Data Corruption。Simulator failure 单列。</t>
+          <t>6) 最终结局分为 Masked、Detected-contained、Data Corruption、Crash、Timeout，另列 Simulator failure。SDC 是 Hardware RAS 全程静默时的错误结果总类：SDC = RAS-silent Data Corruption + RAS-silent Crash + RAS-silent Timeout。Crash、Timeout、Data Corruption 仅是最终表现形式；OS 或 Application 检出不排除 SDC。Masked 与 Simulator failure 不计入 SDC；离线 oracle 不算运行时检测。</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6422,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>SDC=None且Data Corruption；五类结局+Simulator failure=Activated；首检四类=可分析Activated</t>
+          <t>只要 Hardware RAS 任意时点检出数为 0，Data Corruption、Crash、Timeout 均计入 SDC；OS/Application 首检不排除 SDC；Masked 与 Simulator failure 不计入 SDC；五类最终结局+Simulator failure与Activated按现有激活口径核对；首检四类=可分析Activated</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6753,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>合法目标出现率=eligible/attempted；故障激活率=activated/eligible；可分析activated=activated-post_activation_simulator_failure；SDC率=SDC/可分析activated</t>
+          <t>合法目标出现率=eligible/attempted；故障激活率=activated/eligible；可分析activated=activated-post_activation_simulator_failure；SDC=RAS-silent Data Corruption+RAS-silent Crash+RAS-silent Timeout；SDC率=SDC/可分析activated</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -6760,7 +6768,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>避免空项和模拟器失败稀释结果</t>
+          <t>检测维度与最终表现维度分开；OS/Application 检出不排除 SDC；模拟器失败不进入 SDC</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -8020,13 +8028,27 @@
         </is>
       </c>
       <c r="P3" s="9" t="n"/>
-      <c r="Q3" s="9" t="n"/>
-      <c r="R3" s="9" t="n"/>
-      <c r="S3" s="9" t="n"/>
-      <c r="T3" s="9" t="n"/>
-      <c r="U3" s="9" t="n"/>
-      <c r="V3" s="9" t="n"/>
-      <c r="W3" s="9" t="n"/>
+      <c r="Q3" s="9" t="n">
+        <v>385</v>
+      </c>
+      <c r="R3" s="9" t="n">
+        <v>385</v>
+      </c>
+      <c r="S3" s="9" t="n">
+        <v>243</v>
+      </c>
+      <c r="T3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="9" t="n">
+        <v>142</v>
+      </c>
+      <c r="W3" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="X3" s="12">
         <f>IF(OR(R3="",R3-AP3&lt;=0),"",AB3/(R3-AP3))</f>
         <v/>
@@ -8037,20 +8059,38 @@
       </c>
       <c r="Z3" s="9" t="inlineStr">
         <is>
-          <t>待执行</t>
-        </is>
-      </c>
-      <c r="AA3" s="9" t="n"/>
-      <c r="AB3" s="9" t="n"/>
-      <c r="AC3" s="9" t="n"/>
-      <c r="AD3" s="9" t="n"/>
-      <c r="AE3" s="9" t="n"/>
-      <c r="AF3" s="9" t="n"/>
+          <t>部分证据/待核对</t>
+        </is>
+      </c>
+      <c r="AA3" s="9" t="inlineStr">
+        <is>
+          <t>[2026-10-12 formal 回填|0201|HEAD 5c200ff→本提交|binary 1a618953|触发=F0等价(cycle1000,max_faults1)|seed 按协议第10条formal派生] 已覆盖子模型:D01-a(opcode/主操作码字段,opcode_bitflip/transient_bit_flip@coremark):attempted 385/activated 385/Masked 243/Crash 142/SDC 0/Hang 0;P_DUE 36.9%[32.2,41.8](pilot 30%,一致)。本行=预登记重点(2401):现仅记录385层,2401扩样待全行子模型(b/c/d)齐后另行规划。未运行子模型:D01-b/c/d。负载注意:W6定义=CoreMark+Embench全集,本证据仅CoreMark→部分证据。证据:runs/formal_D01-F0-W6-a/c0000/results.jsonl;artifacts/formal_D01-F0-W6-a/summary.md;独立审计:主agent全集核验(385 distinct,r0000-r0384,385×f=1)</t>
+        </is>
+      </c>
+      <c r="AB3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="9" t="n">
+        <v>142</v>
+      </c>
+      <c r="AE3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="9" t="n">
+        <v>243</v>
+      </c>
       <c r="AG3" s="9" t="n"/>
       <c r="AH3" s="9" t="n"/>
       <c r="AI3" s="9" t="n"/>
       <c r="AJ3" s="9" t="n"/>
-      <c r="AK3" s="9" t="n"/>
+      <c r="AK3" s="9" t="inlineStr">
+        <is>
+          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
+        </is>
+      </c>
       <c r="AL3" s="12">
         <f>IF(OR(R3="",R3-AP3&lt;=0),"",AO3/(R3-AP3))</f>
         <v/>
@@ -8063,8 +8103,12 @@
         <f>IF(R3="","",SUM(S3:W3)+AP3-R3)</f>
         <v/>
       </c>
-      <c r="AO3" s="9" t="n"/>
-      <c r="AP3" s="9" t="n"/>
+      <c r="AO3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="AQ3" s="27" t="inlineStr">
         <is>
           <t>D01-a opcode/主操作码字段；D01-b 源/目的寄存器字段；D01-c 立即数/移位字段；D01-d 标志与控制字段；每次只翻1 bit</t>
@@ -8941,9 +8985,8 @@
       <c r="W9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X9" s="12">
-        <f>IF(OR(R9="",R9-AP9&lt;=0),"",AB9/(R9-AP9))</f>
-        <v/>
+      <c r="X9" s="41" t="n">
+        <v>0.1896103896103896</v>
       </c>
       <c r="Y9" s="12">
         <f>IFERROR(R9/AR9,0)</f>
@@ -8956,11 +8999,11 @@
       </c>
       <c r="AA9" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:D02-a(同字段相邻双bit,sub_field=bitflip2_adj,decode/coremark):attempted 385/activated 385/Masked 312/Crash 73/SDC 0/Hang 0。负载注意:W6 定义=CoreMark+Embench 全集,本证据仅跑 CoreMark(Embench 未跑)→部分证据。未运行子模型:D02-b/c。证据:runs/formal_D02a_coremark/c0000/results.jsonl;artifacts/formal_D02a_coremark/summary.md</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:D02-a(同字段相邻双bit,sub_field=bitflip2_adj,decode/coremark):attempted 385/activated 385/Masked 312/Crash 73/SDC 73（RAS-silent Crash 73）/Hang 0。负载注意:W6 定义=CoreMark+Embench 全集,本证据仅跑 CoreMark(Embench 未跑)→部分证据。未运行子模型:D02-b/c。证据:runs/formal_D02a_coremark/c0000/results.jsonl;artifacts/formal_D02a_coremark/summary.md；[2026-10-12 SDC口径修正] SDC=73（Data Corruption 0+RAS-silent Crash 73+RAS-silent Timeout 0），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB9" s="9" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="AC9" s="9" t="n">
         <v>0</v>
@@ -8976,20 +9019,22 @@
       </c>
       <c r="AG9" s="9" t="n"/>
       <c r="AH9" s="9" t="n"/>
-      <c r="AI9" s="9" t="n"/>
-      <c r="AJ9" s="9" t="n"/>
+      <c r="AI9" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="AJ9" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="AK9" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL9" s="12">
-        <f>IF(OR(R9="",R9-AP9&lt;=0),"",AO9/(R9-AP9))</f>
-        <v/>
-      </c>
-      <c r="AM9" s="11">
-        <f>IF(R9="","",SUM(AC9:AF9)-(R9-AP9))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL9" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN9" s="11">
         <f>IF(R9="","",SUM(S9:W9)+AP9-R9)</f>
@@ -10477,9 +10522,8 @@
       <c r="W19" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X19" s="12">
-        <f>IF(OR(R19="",R19-AP19&lt;=0),"",AB19/(R19-AP19))</f>
-        <v/>
+      <c r="X19" s="41" t="n">
+        <v>0.1701298701298701</v>
       </c>
       <c r="Y19" s="12">
         <f>IFERROR(R19/AR19,0)</f>
@@ -10492,11 +10536,11 @@
       </c>
       <c r="AA19" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型×2(行内计数为两者合计,分开统计如下):D04-c(src0/src1互换,src_swap,decode/dep_chain):385/385/Masked 310/Crash 75/SDC 0;D04-e(x0注入,x0_sub,decode/dep_chain):385/385/Masked 329/Crash 56/SDC 0。未运行子模型:D04-a/b/d。证据:runs/formal_D04c_depchain/c0000/results.jsonl;runs/formal_D04e_depchain/c0000/results.jsonl;artifacts/formal_D04{c,e}_depchain/summary.md;双通道审计(subagent A)PASS</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型×2(行内计数为两者合计,分开统计如下):D04-c(src0/src1互换,src_swap,decode/dep_chain):385/385/Masked 310/Crash 75/SDC 75（RAS-silent Crash）;D04-e(x0注入,x0_sub,decode/dep_chain):385/385/Masked 329/Crash 56/SDC 56（RAS-silent Crash）。未运行子模型:D04-a/b/d。证据:runs/formal_D04c_depchain/c0000/results.jsonl;runs/formal_D04e_depchain/c0000/results.jsonl;artifacts/formal_D04{c,e}_depchain/summary.md;双通道审计(subagent A)PASS；[2026-10-12 SDC口径修正] SDC=131（Data Corruption 0+RAS-silent Crash 131+RAS-silent Timeout 0），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB19" s="9" t="n">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="AC19" s="9" t="n">
         <v>0</v>
@@ -10512,20 +10556,22 @@
       </c>
       <c r="AG19" s="9" t="n"/>
       <c r="AH19" s="9" t="n"/>
-      <c r="AI19" s="9" t="n"/>
-      <c r="AJ19" s="9" t="n"/>
+      <c r="AI19" s="9" t="n">
+        <v>131</v>
+      </c>
+      <c r="AJ19" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="AK19" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL19" s="12">
-        <f>IF(OR(R19="",R19-AP19&lt;=0),"",AO19/(R19-AP19))</f>
-        <v/>
-      </c>
-      <c r="AM19" s="11">
-        <f>IF(R19="","",SUM(AC19:AF19)-(R19-AP19))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN19" s="11">
         <f>IF(R19="","",SUM(S19:W19)+AP19-R19)</f>
@@ -11264,7 +11310,7 @@
       </c>
       <c r="AA24" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 D05-b(立即数循环移位,imm_rotate,decode)已于非矩阵负载 dep_chain(W4) 完成 385 样本(attempted 385/activated 385/Masked 277/Crash 108/SDC 0;证据:runs/formal_D05b_depchain/c0000/results.jsonl;双通道审计 PASS)。本行矩阵负载 W3 A64-DecodeProbe 未运行(D05 无 W4 行),不关闭本 RunID。</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 D05-b(立即数循环移位,imm_rotate,decode)已于非矩阵负载 dep_chain(W4) 完成 385 样本(attempted 385/activated 385/Masked 277/Crash 108/SDC 108（RAS-silent Crash 108）;证据:runs/formal_D05b_depchain/c0000/results.jsonl;双通道审计 PASS)。本行矩阵负载 W3 A64-DecodeProbe 未运行(D05 无 W4 行),不关闭本 RunID。；[2026-10-12 SDC口径修正] 跨负载证据仅修正分类口径，仍不关闭本RunID</t>
         </is>
       </c>
       <c r="AB24" s="9" t="n"/>
@@ -11418,7 +11464,7 @@
       </c>
       <c r="AA25" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 D05-b(imm_rotate)已于非矩阵负载 dep_chain(W4) 完成 385 样本(Masked 277/Crash 108/SDC 0;证据:runs/formal_D05b_depchain/c0000/results.jsonl)。本行矩阵负载 W6 CoreMark+Embench 未运行,不关闭本 RunID。</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 D05-b(imm_rotate)已于非矩阵负载 dep_chain(W4) 完成 385 样本(Masked 277/Crash 108/SDC 108（RAS-silent Crash 108）;证据:runs/formal_D05b_depchain/c0000/results.jsonl)。本行矩阵负载 W6 CoreMark+Embench 未运行,不关闭本 RunID。；[2026-10-12 SDC口径修正] 跨负载证据仅修正分类口径，仍不关闭本RunID</t>
         </is>
       </c>
       <c r="AB25" s="9" t="n"/>
@@ -16071,9 +16117,8 @@
       <c r="W56" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="X56" s="12">
-        <f>IF(OR(R56="",R56-AP56&lt;=0),"",AB56/(R56-AP56))</f>
-        <v/>
+      <c r="X56" s="41" t="n">
+        <v>0.5826771653543307</v>
       </c>
       <c r="Y56" s="12">
         <f>IFERROR(R56/AR56,0)</f>
@@ -16086,11 +16131,11 @@
       </c>
       <c r="AA56" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:R02-a(同tag相邻双bit,map_bitflip2_adj,rat/dep_chain):attempted 385/activated 382/Masked 162/SDC 4/Crash 215/Hang 3/SimErr 1。守恒注:3 个 Hang 为 f=null(timeout,注入状态不可判定),不激活但计入结局→AN 差额=3 属如实记录;1 个 SimErr(activated 但模拟器断,不入 n_valid)。未运行子模型:R02-b。证据:runs/formal_R02a_depchain/c0000/results.jsonl;artifacts/formal_R02a_depchain/summary.md</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:R02-a(同tag相邻双bit,map_bitflip2_adj,rat/dep_chain):attempted 385/activated 382/Masked 162/SDC 222（Data Corruption 4+RAS-silent Crash 215+RAS-silent Timeout 3）/Crash 215/Hang 3/SimErr 1。守恒注:3 个 Hang 为 f=null(timeout,注入状态不可判定),不激活但计入结局→AN 差额=3 属如实记录;1 个 SimErr(activated 但模拟器断,不入 n_valid)。未运行子模型:R02-b。证据:runs/formal_R02a_depchain/c0000/results.jsonl;artifacts/formal_R02a_depchain/summary.md；[2026-10-12 SDC口径修正] SDC=222（Data Corruption 4+RAS-silent Crash 215+RAS-silent Timeout 3），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB56" s="9" t="n">
-        <v>4</v>
+        <v>222</v>
       </c>
       <c r="AC56" s="9" t="n">
         <v>0</v>
@@ -16099,27 +16144,29 @@
         <v>215</v>
       </c>
       <c r="AE56" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AF56" s="9" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="AG56" s="9" t="n"/>
       <c r="AH56" s="9" t="n"/>
-      <c r="AI56" s="9" t="n"/>
-      <c r="AJ56" s="9" t="n"/>
+      <c r="AI56" s="9" t="n">
+        <v>215</v>
+      </c>
+      <c r="AJ56" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="AK56" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL56" s="12">
-        <f>IF(OR(R56="",R56-AP56&lt;=0),"",AO56/(R56-AP56))</f>
-        <v/>
-      </c>
-      <c r="AM56" s="11">
-        <f>IF(R56="","",SUM(AC56:AF56)-(R56-AP56))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL56" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM56" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN56" s="11">
         <f>IF(R56="","",SUM(S56:W56)+AP56-R56)</f>
@@ -16707,9 +16754,8 @@
       <c r="W60" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X60" s="12">
-        <f>IF(OR(R60="",R60-AP60&lt;=0),"",AB60/(R60-AP60))</f>
-        <v/>
+      <c r="X60" s="41" t="n">
+        <v>0.2103896103896104</v>
       </c>
       <c r="Y60" s="12">
         <f>IFERROR(R60/AR60,0)</f>
@@ -16722,11 +16768,11 @@
       </c>
       <c r="AA60" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:R03-c(src0/src1 tag互换,src_tag_swap,rat/dep_chain):attempted 385/activated 385/Masked 304/Crash 81/SDC 0/Hang 0。未运行子模型:R03-a/b。证据:runs/formal_R03c_depchain/c0000/results.jsonl;artifacts/formal_R03c_depchain/summary.md;双通道审计(subagent A)PASS</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:R03-c(src0/src1 tag互换,src_tag_swap,rat/dep_chain):attempted 385/activated 385/Masked 304/Crash 81/SDC 81（RAS-silent Crash 81）/Hang 0。未运行子模型:R03-a/b。证据:runs/formal_R03c_depchain/c0000/results.jsonl;artifacts/formal_R03c_depchain/summary.md;双通道审计(subagent A)PASS；[2026-10-12 SDC口径修正] SDC=81（Data Corruption 0+RAS-silent Crash 81+RAS-silent Timeout 0），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB60" s="9" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="AC60" s="9" t="n">
         <v>0</v>
@@ -16742,20 +16788,22 @@
       </c>
       <c r="AG60" s="9" t="n"/>
       <c r="AH60" s="9" t="n"/>
-      <c r="AI60" s="9" t="n"/>
-      <c r="AJ60" s="9" t="n"/>
+      <c r="AI60" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="AJ60" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="AK60" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL60" s="12">
-        <f>IF(OR(R60="",R60-AP60&lt;=0),"",AO60/(R60-AP60))</f>
-        <v/>
-      </c>
-      <c r="AM60" s="11">
-        <f>IF(R60="","",SUM(AC60:AF60)-(R60-AP60))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL60" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM60" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN60" s="11">
         <f>IF(R60="","",SUM(S60:W60)+AP60-R60)</f>
@@ -23493,9 +23541,8 @@
       <c r="W105" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X105" s="12">
-        <f>IF(OR(R105="",R105-AP105&lt;=0),"",AB105/(R105-AP105))</f>
-        <v/>
+      <c r="X105" s="41" t="n">
+        <v>0</v>
       </c>
       <c r="Y105" s="12">
         <f>IFERROR(R105/AR105,0)</f>
@@ -23508,7 +23555,7 @@
       </c>
       <c r="AA105" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:B02-a(同字段相邻双bit,pc_bitflip2_adj,rob/rob_fill):attempted 385/activated 385/Masked 385/Crash 0/SDC 0/Hang 0(100% Masked)。未运行子模型:B02-b。证据:runs/formal_B02a_robfill/c0000/results.jsonl;artifacts/formal_B02a_robfill/summary.md</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:B02-a(同字段相邻双bit,pc_bitflip2_adj,rob/rob_fill):attempted 385/activated 385/Masked 385/Crash 0/SDC 0/Hang 0(100% Masked)。未运行子模型:B02-b。证据:runs/formal_B02a_robfill/c0000/results.jsonl;artifacts/formal_B02a_robfill/summary.md；[2026-10-12 SDC口径修正] SDC=0（Data Corruption 0+RAS-silent Crash 0+RAS-silent Timeout 0），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB105" s="9" t="n">
@@ -23528,20 +23575,22 @@
       </c>
       <c r="AG105" s="9" t="n"/>
       <c r="AH105" s="9" t="n"/>
-      <c r="AI105" s="9" t="n"/>
-      <c r="AJ105" s="9" t="n"/>
+      <c r="AI105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ105" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="AK105" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL105" s="12">
-        <f>IF(OR(R105="",R105-AP105&lt;=0),"",AO105/(R105-AP105))</f>
-        <v/>
-      </c>
-      <c r="AM105" s="11">
-        <f>IF(R105="","",SUM(AC105:AF105)-(R105-AP105))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL105" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM105" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN105" s="11">
         <f>IF(R105="","",SUM(S105:W105)+AP105-R105)</f>
@@ -31480,7 +31529,7 @@
       </c>
       <c r="AA158" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 FD02-a(同字段相邻双bit,fp_bitflip2_adj,decode)已于非矩阵负载 polybench/gemm 完成 385 样本(attempted 385/activated 385/Masked 166/Crash 143/SDC 76;证据:runs/formal_FD02a_gemm/c0000/results.jsonl)。本行矩阵负载 W8 FP-ScalarProbe 未运行,不关闭本 RunID。</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 FD02-a(同字段相邻双bit,fp_bitflip2_adj,decode)已于非矩阵负载 polybench/gemm 完成 385 样本(attempted 385/activated 385/Masked 166/Crash 143/SDC 219（Data Corruption 76+RAS-silent Crash 143）;证据:runs/formal_FD02a_gemm/c0000/results.jsonl)。本行矩阵负载 W8 FP-ScalarProbe 未运行,不关闭本 RunID。；[2026-10-12 SDC口径修正] 跨负载证据仅修正分类口径，仍不关闭本RunID</t>
         </is>
       </c>
       <c r="AB158" s="9" t="n"/>
@@ -31634,7 +31683,7 @@
       </c>
       <c r="AA159" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 FD02-a 同上(gemm 385 样本,Masked 166/Crash 143/SDC 76)。本行矩阵负载 W9 NEON-LaneProbe 未运行,不关闭本 RunID。证据:runs/formal_FD02a_gemm/c0000/results.jsonl。</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 跨负载部分证据备注:子模型 FD02-a 同上(gemm 385 样本,Masked 166/Crash 143/SDC 219（Data Corruption 76+RAS-silent Crash 143）)。本行矩阵负载 W9 NEON-LaneProbe 未运行,不关闭本 RunID。证据:runs/formal_FD02a_gemm/c0000/results.jsonl。；[2026-10-12 SDC口径修正] 跨负载证据仅修正分类口径，仍不关闭本RunID</t>
         </is>
       </c>
       <c r="AB159" s="9" t="n"/>
@@ -39287,9 +39336,8 @@
       <c r="W210" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="X210" s="12">
-        <f>IF(OR(R210="",R210-AP210&lt;=0),"",AB210/(R210-AP210))</f>
-        <v/>
+      <c r="X210" s="41" t="n">
+        <v>0.1707317073170732</v>
       </c>
       <c r="Y210" s="12">
         <f>IFERROR(R210/AR210,0)</f>
@@ -39302,11 +39350,11 @@
       </c>
       <c r="AA210" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:FR02-a(同tag相邻双bit,map_bitflip2_adj_vec,rat)。[recount 修正口径,2026-10-10 审计提交 0244e9c]attempted 650/activated 328/Masked 275/SDC 45/Crash 8/Hang 3/Inactive 322;假激活 49 条已剔除(旧口径 390/380 作废)。formal 未达标:activated 328 &lt; 385,差 57。负载注意:证据负载为 dep_chain_vec(非 W9 NEON-LaneProbe 定义,W9 探针未开发)→部分证据,FR02-b 未运行。守恒注:3 个 Hang 为 f=null→AN 差额=3 属如实记录。补量待 FP/SIMD Rename 单元按矩阵负载执行。证据:runs/formal_FR02_dcv/c0000/results.jsonl;docs/gem5-fi/ooo/fr02-recount-audit-2026-10-10.md;fr02-correction-overlay-2026-10-10.json</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:FR02-a(同tag相邻双bit,map_bitflip2_adj_vec,rat)。[recount 修正口径,2026-10-10 审计提交 0244e9c]attempted 650/activated 328/Masked 275/SDC 56（Data Corruption 45+RAS-silent Crash 8+RAS-silent Timeout 3）/Crash 8/Hang 3/Inactive 322;假激活 49 条已剔除(旧口径 390/380 作废)。formal 未达标:activated 328 &lt; 385,差 57。负载注意:证据负载为 dep_chain_vec(非 W9 NEON-LaneProbe 定义,W9 探针未开发)→部分证据,FR02-b 未运行。守恒注:3 个 Hang 为 f=null→AN 差额=3 属如实记录。补量待 FP/SIMD Rename 单元按矩阵负载执行。证据:runs/formal_FR02_dcv/c0000/results.jsonl;docs/gem5-fi/ooo/fr02-recount-audit-2026-10-10.md;fr02-correction-overlay-2026-10-10.json；[2026-10-12 SDC口径修正] SDC=56（Data Corruption 45+RAS-silent Crash 8+RAS-silent Timeout 3），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB210" s="9" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="AC210" s="9" t="n">
         <v>0</v>
@@ -39315,27 +39363,29 @@
         <v>8</v>
       </c>
       <c r="AE210" s="9" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="AF210" s="9" t="n">
-        <v>275</v>
+        <v>320</v>
       </c>
       <c r="AG210" s="9" t="n"/>
       <c r="AH210" s="9" t="n"/>
-      <c r="AI210" s="9" t="n"/>
-      <c r="AJ210" s="9" t="n"/>
+      <c r="AI210" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ210" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="AK210" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL210" s="12">
-        <f>IF(OR(R210="",R210-AP210&lt;=0),"",AO210/(R210-AP210))</f>
-        <v/>
-      </c>
-      <c r="AM210" s="11">
-        <f>IF(R210="","",SUM(AC210:AF210)-(R210-AP210))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL210" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM210" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN210" s="11">
         <f>IF(R210="","",SUM(S210:W210)+AP210-R210)</f>
@@ -47427,9 +47477,8 @@
       <c r="W264" s="9" t="n">
         <v>102</v>
       </c>
-      <c r="X264" s="12">
-        <f>IF(OR(R264="",R264-AP264&lt;=0),"",AB264/(R264-AP264))</f>
-        <v/>
+      <c r="X264" s="41" t="n">
+        <v>0.2649350649350649</v>
       </c>
       <c r="Y264" s="12">
         <f>IFERROR(R264/AR264,0)</f>
@@ -47442,11 +47491,11 @@
       </c>
       <c r="AA264" s="9" t="inlineStr">
         <is>
-          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:FB02-a(同字段相邻双bit,destid_bitflip2_adj_vec,rob/gemm):attempted 385/activated 385/Masked 283/Hang 102/Crash 0/SDC 0。负载注意:W10 定义=PolyBench 五内核(gemm/2mm/lu/cholesky/jacobi-2d),本证据仅跑 gemm(1/5)→部分证据。未运行子模型:FB02-b。证据:runs/formal_FB02_gemm/c0000/results.jsonl;artifacts/formal_FB02_gemm/summary.md</t>
+          <t>[2026-10-12 过渡回填|0201(huawei0201,172.168.178.81)|HEAD bf3d284|binary 1a618953|触发=F0等价(cycle1000 warm-up,max_faults1,首个eligible)] 已覆盖子模型:FB02-a(同字段相邻双bit,destid_bitflip2_adj_vec,rob/gemm):attempted 385/activated 385/Masked 283/Hang 102/Crash 0/SDC 102（RAS-silent Timeout 102）。负载注意:W10 定义=PolyBench 五内核(gemm/2mm/lu/cholesky/jacobi-2d),本证据仅跑 gemm(1/5)→部分证据。未运行子模型:FB02-b。证据:runs/formal_FB02_gemm/c0000/results.jsonl;artifacts/formal_FB02_gemm/summary.md；[2026-10-12 SDC口径修正] SDC=102（Data Corruption 0+RAS-silent Crash 0+RAS-silent Timeout 102），原始结局计数不变</t>
         </is>
       </c>
       <c r="AB264" s="9" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="AC264" s="9" t="n">
         <v>0</v>
@@ -47462,20 +47511,22 @@
       </c>
       <c r="AG264" s="9" t="n"/>
       <c r="AH264" s="9" t="n"/>
-      <c r="AI264" s="9" t="n"/>
-      <c r="AJ264" s="9" t="n"/>
+      <c r="AI264" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ264" s="9" t="n">
+        <v>102</v>
+      </c>
       <c r="AK264" s="9" t="inlineStr">
         <is>
-          <t>SE口径推定首检:Masked→None;SDC→Application(oracle校验和);Crash/Hang→OS(abort/timeout看门狗);硬件RAS=0(B0无ECC/parity)</t>
-        </is>
-      </c>
-      <c r="AL264" s="12">
-        <f>IF(OR(R264="",R264-AP264&lt;=0),"",AO264/(R264-AP264))</f>
-        <v/>
-      </c>
-      <c r="AM264" s="11">
-        <f>IF(R264="","",SUM(AC264:AF264)-(R264-AP264))</f>
-        <v/>
+          <t>SE口径首检：Masked及仅由离线oracle发现的Data Corruption→None；架构Crash/已归因Timeout→OS；Hardware RAS任意时点=0（B0无ECC/parity）。OS/Application检出不排除SDC。</t>
+        </is>
+      </c>
+      <c r="AL264" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM264" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="AN264" s="11">
         <f>IF(R264="","",SUM(S264:W264)+AP264-R264)</f>

</xml_diff>